<commit_message>
Barrio Obrero: empleo (PERSONAL_O) en Desarrollo Economico + fila educacion 2026 informativa + Excel sin nota_estado
- DE ahora con 4 componentes (establecimientos+ingresos+activo+EMPLEO), igual que
  Ciudad Paraiso: empleo del geojson 2025 (PERSONAL_O) mapeado por numeroInscrito y
  sumado sobre el stock activo por anio. Empleo 1710/1762/1785/1750. ITT: 51.7/57.7/56.9/73.2.
- Hoja Educacion: fila 2026 informativa (matricula 867, repitentes 104, corte marzo,
  NO entra al ITT; desercion NaN por SIMPADE no cerrado).
- Excel: columna interna nota_estado eliminada de todas las hojas.
</commit_message>
<xml_diff>
--- a/outputs/itt_barrio_obrero/ITT_Barrio_Obrero_Consolidado.xlsx
+++ b/outputs/itt_barrio_obrero/ITT_Barrio_Obrero_Consolidado.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -469,7 +469,6 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,11 +512,6 @@
           <t>nivel</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>nota_estado</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -536,19 +530,14 @@
         <v>60.7</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>52.47</v>
+        <v>60.18</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>50.55</v>
+        <v>51.7</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Consolidacion</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
         </is>
       </c>
     </row>
@@ -569,19 +558,14 @@
         <v>64.3</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>96.34999999999999</v>
+        <v>93.72</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>58.08</v>
+        <v>57.69</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Consolidacion</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
         </is>
       </c>
     </row>
@@ -602,19 +586,14 @@
         <v>63</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>67.93000000000001</v>
+        <v>72.69</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>56.13</v>
+        <v>56.85</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Consolidacion</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
         </is>
       </c>
     </row>
@@ -635,19 +614,14 @@
         <v>57.2</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>66.67</v>
+        <v>71.31</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>72.45</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Parcial (no comparable)</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Parcial Q1-Q2 | DesSocial y DesEco referenciales</t>
         </is>
       </c>
     </row>
@@ -712,7 +686,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>30.13</v>
+        <v>31.28</v>
       </c>
       <c r="E2" s="2" t="b">
         <v>0</v>
@@ -731,7 +705,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>27.43</v>
+        <v>28.58</v>
       </c>
       <c r="E3" s="2" t="b">
         <v>0</v>
@@ -750,7 +724,7 @@
         <v>3</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>48.26</v>
+        <v>49.41</v>
       </c>
       <c r="E4" s="2" t="b">
         <v>0</v>
@@ -769,7 +743,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>30.13</v>
+        <v>31.28</v>
       </c>
       <c r="E5" s="2" t="b">
         <v>0</v>
@@ -788,7 +762,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>35.37</v>
+        <v>34.97</v>
       </c>
       <c r="E6" s="2" t="b">
         <v>0</v>
@@ -807,7 +781,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>56.2</v>
+        <v>55.81</v>
       </c>
       <c r="E7" s="2" t="b">
         <v>0</v>
@@ -826,7 +800,7 @@
         <v>3</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46.94</v>
+        <v>46.54</v>
       </c>
       <c r="E8" s="2" t="b">
         <v>0</v>
@@ -845,7 +819,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>42.7</v>
+        <v>42.31</v>
       </c>
       <c r="E9" s="2" t="b">
         <v>0</v>
@@ -864,7 +838,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>38.35</v>
+        <v>39.06</v>
       </c>
       <c r="E10" s="2" t="b">
         <v>0</v>
@@ -883,7 +857,7 @@
         <v>2</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>36.77</v>
+        <v>37.49</v>
       </c>
       <c r="E11" s="2" t="b">
         <v>0</v>
@@ -902,7 +876,7 @@
         <v>3</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>36.77</v>
+        <v>37.49</v>
       </c>
       <c r="E12" s="2" t="b">
         <v>0</v>
@@ -921,7 +895,7 @@
         <v>4</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>39.47</v>
+        <v>40.19</v>
       </c>
       <c r="E13" s="2" t="b">
         <v>0</v>
@@ -940,7 +914,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>50.12</v>
+        <v>50.82</v>
       </c>
       <c r="E14" s="3" t="b">
         <v>1</v>
@@ -959,7 +933,7 @@
         <v>2</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>35.85</v>
+        <v>36.55</v>
       </c>
       <c r="E15" s="3" t="b">
         <v>1</v>
@@ -978,7 +952,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>35.85</v>
+        <v>36.55</v>
       </c>
       <c r="E16" s="3" t="b">
         <v>1</v>
@@ -997,7 +971,7 @@
         <v>4</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>35.85</v>
+        <v>36.55</v>
       </c>
       <c r="E17" s="3" t="b">
         <v>1</v>
@@ -1014,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1023,7 +997,6 @@
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1057,11 +1030,6 @@
           <t>score_seguridad</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>nota_estado</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1082,11 +1050,6 @@
       <c r="F2" s="2" t="n">
         <v>66.11</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1107,11 +1070,6 @@
       <c r="F3" s="2" t="n">
         <v>36.88</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1132,11 +1090,6 @@
       <c r="F4" s="2" t="n">
         <v>33.23</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -1156,11 +1109,6 @@
       </c>
       <c r="F5" s="3" t="n">
         <v>66.81</v>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Parcial Q1-Q2</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1174,7 +1122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1185,7 +1133,6 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1229,11 +1176,6 @@
           <t>score_movilidad</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>nota_estado</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1260,11 +1202,6 @@
       <c r="H2" s="2" t="n">
         <v>23.96</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1291,11 +1228,6 @@
       <c r="H3" s="2" t="n">
         <v>57.99</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1322,11 +1254,6 @@
       <c r="H4" s="2" t="n">
         <v>80.56</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -1352,11 +1279,6 @@
       </c>
       <c r="H5" s="3" t="n">
         <v>84.38</v>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Parcial Q1-Q2</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1370,7 +1292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1381,7 +1303,6 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1425,11 +1346,6 @@
           <t>score_cohesion</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>nota_estado</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1456,11 +1372,6 @@
       <c r="H2" s="2" t="n">
         <v>55.23</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1487,11 +1398,6 @@
       <c r="H3" s="2" t="n">
         <v>82.13</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1518,11 +1424,6 @@
       <c r="H4" s="2" t="n">
         <v>38.01</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -1548,11 +1449,6 @@
       </c>
       <c r="H5" s="3" t="n">
         <v>84.88</v>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Parcial Q1-Q2</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1566,7 +1462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1575,7 +1471,6 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1609,11 +1504,6 @@
           <t>score_entorno_u</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>nota_estado</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1634,11 +1524,6 @@
       <c r="F2" s="2" t="n">
         <v>60.7</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Real (NDVI anual + DAGMA)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1659,11 +1544,6 @@
       <c r="F3" s="2" t="n">
         <v>64.3</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Real (NDVI anual + DAGMA)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1684,11 +1564,6 @@
       <c r="F4" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Real (NDVI anual + DAGMA)</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -1708,11 +1583,6 @@
       </c>
       <c r="F5" s="3" t="n">
         <v>57.2</v>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Real (NDVI anual + DAGMA)</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1726,7 +1596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1736,7 +1606,7 @@
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1777,7 +1647,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>nota_estado</t>
+          <t>observacion</t>
         </is>
       </c>
     </row>
@@ -1803,11 +1673,7 @@
       <c r="G2" s="2" t="n">
         <v>13.7</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Real (SIMAT + SIMPADE)</t>
-        </is>
-      </c>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1831,11 +1697,7 @@
       <c r="G3" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Real (SIMAT + SIMPADE)</t>
-        </is>
-      </c>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1859,9 +1721,27 @@
       <c r="G4" s="2" t="n">
         <v>29.8</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Real (SIMAT + SIMPADE)</t>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>867</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Corte marzo 2026 - informativo, NO entra al ITT (anio no cerrado, sin desercion SIMPADE)</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1887,11 +1767,12 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1937,27 +1818,32 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>empleo_personas</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>score_establecimientos</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>score_ingresos</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>score_activo_total</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>score_empleo</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>score_des_eco</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>nota_estado</t>
         </is>
       </c>
     </row>
@@ -1989,21 +1875,22 @@
         <v>25.7</v>
       </c>
       <c r="I2" s="2" t="n">
+        <v>1710</v>
+      </c>
+      <c r="J2" s="2" t="n">
         <v>82.02</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="K2" s="2" t="n">
         <v>75.40000000000001</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="L2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" s="2" t="n">
-        <v>52.47</v>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Real (stock activo consolidado)</t>
-        </is>
+      <c r="M2" s="2" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>60.18</v>
       </c>
     </row>
     <row r="3">
@@ -2034,21 +1921,22 @@
         <v>25.72</v>
       </c>
       <c r="I3" s="2" t="n">
+        <v>1762</v>
+      </c>
+      <c r="J3" s="2" t="n">
         <v>89.34</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="K3" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="L3" s="2" t="n">
         <v>99.7</v>
       </c>
-      <c r="L3" s="2" t="n">
-        <v>96.34999999999999</v>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Real (stock activo consolidado)</t>
-        </is>
+      <c r="M3" s="2" t="n">
+        <v>85.84</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>93.72</v>
       </c>
     </row>
     <row r="4">
@@ -2079,21 +1967,22 @@
         <v>25.72</v>
       </c>
       <c r="I4" s="2" t="n">
+        <v>1785</v>
+      </c>
+      <c r="J4" s="2" t="n">
         <v>96.67</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="K4" s="2" t="n">
         <v>22.8</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="L4" s="2" t="n">
         <v>84.31999999999999</v>
       </c>
-      <c r="L4" s="2" t="n">
-        <v>67.93000000000001</v>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>Real (stock activo consolidado)</t>
-        </is>
+      <c r="M4" s="2" t="n">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>72.69</v>
       </c>
     </row>
     <row r="5">
@@ -2124,21 +2013,22 @@
         <v>25.72</v>
       </c>
       <c r="I5" s="3" t="n">
+        <v>1750</v>
+      </c>
+      <c r="J5" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="K5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="L5" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="L5" s="3" t="n">
-        <v>66.67</v>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Real (stock activo consolidado; 2026 parcial, no comparable)</t>
-        </is>
+      <c r="M5" s="3" t="n">
+        <v>85.25</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>71.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Barrio Obrero: elimina columna interna 'parcial' del Excel (uso interno, no en el entregable)
</commit_message>
<xml_diff>
--- a/outputs/itt_barrio_obrero/ITT_Barrio_Obrero_Consolidado.xlsx
+++ b/outputs/itt_barrio_obrero/ITT_Barrio_Obrero_Consolidado.xlsx
@@ -636,14 +636,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -667,11 +666,6 @@
           <t>ITT</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>parcial</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -688,9 +682,6 @@
       <c r="D2" s="2" t="n">
         <v>31.28</v>
       </c>
-      <c r="E2" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -707,9 +698,6 @@
       <c r="D3" s="2" t="n">
         <v>28.58</v>
       </c>
-      <c r="E3" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -726,9 +714,6 @@
       <c r="D4" s="2" t="n">
         <v>49.41</v>
       </c>
-      <c r="E4" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -745,9 +730,6 @@
       <c r="D5" s="2" t="n">
         <v>31.28</v>
       </c>
-      <c r="E5" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -764,9 +746,6 @@
       <c r="D6" s="2" t="n">
         <v>34.97</v>
       </c>
-      <c r="E6" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -783,9 +762,6 @@
       <c r="D7" s="2" t="n">
         <v>55.81</v>
       </c>
-      <c r="E7" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -802,9 +778,6 @@
       <c r="D8" s="2" t="n">
         <v>46.54</v>
       </c>
-      <c r="E8" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -821,9 +794,6 @@
       <c r="D9" s="2" t="n">
         <v>42.31</v>
       </c>
-      <c r="E9" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -840,9 +810,6 @@
       <c r="D10" s="2" t="n">
         <v>39.06</v>
       </c>
-      <c r="E10" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -859,9 +826,6 @@
       <c r="D11" s="2" t="n">
         <v>37.49</v>
       </c>
-      <c r="E11" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -878,9 +842,6 @@
       <c r="D12" s="2" t="n">
         <v>37.49</v>
       </c>
-      <c r="E12" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -897,9 +858,6 @@
       <c r="D13" s="2" t="n">
         <v>40.19</v>
       </c>
-      <c r="E13" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -916,9 +874,6 @@
       <c r="D14" s="3" t="n">
         <v>50.82</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -935,9 +890,6 @@
       <c r="D15" s="3" t="n">
         <v>36.55</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -954,9 +906,6 @@
       <c r="D16" s="3" t="n">
         <v>36.55</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -972,9 +921,6 @@
       </c>
       <c r="D17" s="3" t="n">
         <v>36.55</v>
-      </c>
-      <c r="E17" s="3" t="b">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Barrio Obrero: NDVI actualizado al poligono completo (cubre 100%) + los NDVI de la esquina pasan a V1
- Nuevos rasters barrio_obrero_nuevo_ndvi_* cubren todo el poligono (antes el NDVI
  solo cubria ~27%, una esquina = zona V1). Los antiguos se mueven a NDVI_Barrio_Obrero_v1/.
- Notebook: EU-1 y overlays NDVI usan busqueda flexible por año (_ndvi_tif glob).
- Entorno Urbano recalculado con NDVI real del barrio: score 30.6/32.7/32.4/31.7 (antes
  ~60, sesgado por medir solo la esquina verde). ITT: 46.6/52.3/51.6/68.8 (2026 parcial).
</commit_message>
<xml_diff>
--- a/outputs/itt_barrio_obrero/ITT_Barrio_Obrero_Consolidado.xlsx
+++ b/outputs/itt_barrio_obrero/ITT_Barrio_Obrero_Consolidado.xlsx
@@ -527,13 +527,13 @@
         <v>48.61</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>60.7</v>
+        <v>30.6</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>60.18</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>51.7</v>
+        <v>46.59</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -555,13 +555,13 @@
         <v>52.55</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>64.3</v>
+        <v>32.7</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>93.72</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>57.69</v>
+        <v>52.31</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -583,13 +583,13 @@
         <v>44.95</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>63</v>
+        <v>32.4</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>72.69</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>56.85</v>
+        <v>51.65</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -611,13 +611,13 @@
         <v>84.88</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>57.2</v>
+        <v>31.7</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>71.31</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>73.15000000000001</v>
+        <v>68.81</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>31.28</v>
+        <v>26.16</v>
       </c>
     </row>
     <row r="3">
@@ -696,7 +696,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>28.58</v>
+        <v>23.46</v>
       </c>
     </row>
     <row r="4">
@@ -712,7 +712,7 @@
         <v>3</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>49.41</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="5">
@@ -728,7 +728,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>31.28</v>
+        <v>26.16</v>
       </c>
     </row>
     <row r="6">
@@ -744,7 +744,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>34.97</v>
+        <v>29.6</v>
       </c>
     </row>
     <row r="7">
@@ -760,7 +760,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>55.81</v>
+        <v>50.43</v>
       </c>
     </row>
     <row r="8">
@@ -776,7 +776,7 @@
         <v>3</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46.54</v>
+        <v>41.17</v>
       </c>
     </row>
     <row r="9">
@@ -792,7 +792,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>42.31</v>
+        <v>36.93</v>
       </c>
     </row>
     <row r="10">
@@ -808,7 +808,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>39.06</v>
+        <v>33.86</v>
       </c>
     </row>
     <row r="11">
@@ -824,7 +824,7 @@
         <v>2</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>37.49</v>
+        <v>32.29</v>
       </c>
     </row>
     <row r="12">
@@ -840,7 +840,7 @@
         <v>3</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>37.49</v>
+        <v>32.29</v>
       </c>
     </row>
     <row r="13">
@@ -856,7 +856,7 @@
         <v>4</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>40.19</v>
+        <v>34.99</v>
       </c>
     </row>
     <row r="14">
@@ -872,7 +872,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>50.82</v>
+        <v>46.49</v>
       </c>
     </row>
     <row r="15">
@@ -888,7 +888,7 @@
         <v>2</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>36.55</v>
+        <v>32.21</v>
       </c>
     </row>
     <row r="16">
@@ -904,7 +904,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>36.55</v>
+        <v>32.21</v>
       </c>
     </row>
     <row r="17">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>36.55</v>
+        <v>32.21</v>
       </c>
     </row>
   </sheetData>
@@ -1456,19 +1456,19 @@
         <v>2023</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.0687</v>
+        <v>0.0579</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>6.4</v>
+        <v>4.9</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>5154</v>
+        <v>19130</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>108.8</v>
+        <v>22.4</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>60.7</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="3">
@@ -1476,19 +1476,19 @@
         <v>2024</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.0809</v>
+        <v>0.0769</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>8.6</v>
+        <v>6.2</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6938</v>
+        <v>24285</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>108.8</v>
+        <v>22.4</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>64.3</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="4">
@@ -1496,19 +1496,19 @@
         <v>2025</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.0804</v>
+        <v>0.0728</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>7.8</v>
+        <v>6</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>6245</v>
+        <v>23294</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>108.8</v>
+        <v>22.4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>63</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="5">
@@ -1516,19 +1516,19 @@
         <v>2026</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.0688</v>
+        <v>0.0717</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>3469</v>
+        <v>21906</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>108.8</v>
+        <v>22.4</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>57.2</v>
+        <v>31.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>